<commit_message>
fix(gran-agregado): restore dynamic formula in H14/H15 and eliminate duplicated operator in G10
</commit_message>
<xml_diff>
--- a/app/templates/Subir auditoria/Subir Agregados/1-INF.-N-000-26-AG19-GRAN.-V10.xlsx
+++ b/app/templates/Subir auditoria/Subir Agregados/1-INF.-N-000-26-AG19-GRAN.-V10.xlsx
@@ -38651,10 +38651,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G10" s="470">
-        <f>+FORMATO!H11</f>
-        <v>0</v>
-      </c>
+      <c r="G10" s="470"/>
       <c r="H10" s="470"/>
       <c r="I10" s="470"/>
       <c r="J10" s="470"/>
@@ -38749,7 +38746,7 @@
         <v>285</v>
       </c>
       <c r="H14" s="538">
-        <f>+FORMATO!D35</f>
+        <f>+IF(C10="Global",FORMATO!D21,FORMATO!D35)</f>
         <v>0</v>
       </c>
       <c r="I14" s="442">
@@ -38783,7 +38780,7 @@
         <v>286</v>
       </c>
       <c r="H15" s="539">
-        <f>+FORMATO!D37</f>
+        <f>+IF(C10="Global",FORMATO!D22,FORMATO!D36)</f>
         <v>0</v>
       </c>
       <c r="I15" s="444">

</xml_diff>